<commit_message>
Phase 08: review round 1 - texts DOC-097 to DOC-120 rewritten by hand with distinct layouts, dataset rebuilt, blind second pass on the 24 (G2)
</commit_message>
<xml_diff>
--- a/evals/datasets/document_extraction/files/DOC-101.xlsx
+++ b/evals/datasets/document_extraction/files/DOC-101.xlsx
@@ -413,27 +413,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ventas@dissanorte.example.com</t>
+          <t>INVOICE</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>F-67987</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Invoice F-67987</t>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ventas@dissanorte.example.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Issue date</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -445,7 +455,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Order</t>
+          <t>Purchase order</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -457,73 +467,102 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Unit price</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Amount EUR</t>
+          <t>EUR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Plastic medicine cups 30 ml</t>
+          <t>Item or code</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>Unit price</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14.88</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>URN-CUP-100</t>
+          <t>Plastic medicine cups 30 ml</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11.46</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>573.00</t>
+          <t>14.88</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Handling charge: 26.94 EUR</t>
+          <t>URN-CUP-100</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>11.46</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>573.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Handling fee</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>26.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>614.82</t>
         </is>
       </c>
     </row>

</xml_diff>